<commit_message>
Publish workbenches for 2026-10-19
</commit_message>
<xml_diff>
--- a/docs/downloads/经营分_津河省区__唐山北片区_2026-10-19.xlsx
+++ b/docs/downloads/经营分_津河省区__唐山北片区_2026-10-19.xlsx
@@ -12,7 +12,7 @@
     <sheet name="匹配异常" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'门店经营分'!$A$1:$V$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'门店经营分'!$A$1:$V$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'匹配异常'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1020,20 +1020,24 @@
           <t>唐山北片区</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>唐山市</t>
+        </is>
+      </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>6970807765576976396</t>
+          <t>7649552788984170539</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>喆啡酒店（唐山北大麦广场店）</t>
+          <t>维也纳酒店(滦州市火车站店)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>喆啡酒店(唐山北大麦广场店)</t>
+          <t>维也纳酒店(滦州市火车站店)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1042,18 +1046,18 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>稳房源,提质量,拿收益</t>
+          <t>搭门店,稳房源,提质量,附加分,拿收益</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L6" t="n">
         <v>10</v>
@@ -1065,19 +1069,19 @@
         <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="P6" t="n">
         <v>30</v>
       </c>
       <c r="Q6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R6" t="n">
         <v>30</v>
       </c>
       <c r="S6" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T6" t="n">
         <v>20</v>
@@ -1104,36 +1108,32 @@
           <t>唐山北片区</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>唐山市</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>7102768023395633189</t>
+          <t>6970807765576976396</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>派酒店（唐山迁西北岸新区店）</t>
+          <t>喆啡酒店（唐山北大麦广场店）</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>派酒店(唐山迁西北岸新区店)</t>
+          <t>喆啡酒店(唐山北大麦广场店)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H7" t="n">
         <v>82</v>
       </c>
       <c r="I7" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1199,17 +1199,17 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>7316515741600417842</t>
+          <t>7102768023395633189</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>白玉兰商务酒店（唐山玉田店）</t>
+          <t>派酒店（唐山迁西北岸新区店）</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>白玉兰酒店(玉田店)</t>
+          <t>派酒店(唐山迁西北岸新区店)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1221,7 +1221,7 @@
         <v>82</v>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
         <v>10</v>
       </c>
       <c r="M8" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N8" t="n">
         <v>30</v>
@@ -1247,7 +1247,7 @@
         <v>30</v>
       </c>
       <c r="Q8" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R8" t="n">
         <v>30</v>
@@ -1287,17 +1287,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>7418029787958282277</t>
+          <t>7316515741600417842</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>麗枫酒店（唐山中心医院店）</t>
+          <t>白玉兰商务酒店（唐山玉田店）</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>麗枫酒店(唐山中心医院店)</t>
+          <t>白玉兰酒店(玉田店)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1309,7 +1309,7 @@
         <v>82</v>
       </c>
       <c r="I9" t="n">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         <v>10</v>
       </c>
       <c r="M9" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="N9" t="n">
         <v>30</v>
@@ -1335,7 +1335,7 @@
         <v>30</v>
       </c>
       <c r="Q9" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R9" t="n">
         <v>30</v>
@@ -1375,17 +1375,17 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>6741041123524954123</t>
+          <t>7418029787958282277</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>希岸酒店唐山北站店</t>
+          <t>麗枫酒店（唐山中心医院店）</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>希岸酒店(唐山北站店)</t>
+          <t>麗枫酒店(唐山中心医院店)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1394,10 +1394,10 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
         <v>30</v>
       </c>
       <c r="Q10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R10" t="n">
         <v>30</v>
@@ -1456,20 +1456,24 @@
           <t>唐山北片区</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>唐山市</t>
+        </is>
+      </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>6601265040777545741</t>
+          <t>6741041123524954123</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>希岸酒店河北玉田店</t>
+          <t>希岸酒店唐山北站店</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>希岸酒店(玉田店)</t>
+          <t>希岸酒店(唐山北站店)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1501,13 +1505,13 @@
         <v>30</v>
       </c>
       <c r="O11" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P11" t="n">
         <v>30</v>
       </c>
       <c r="Q11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R11" t="n">
         <v>30</v>
@@ -1540,24 +1544,20 @@
           <t>唐山北片区</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>唐山市</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>7382896529226336271</t>
+          <t>6601265040777545741</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>维也纳酒店（唐山丰润林荫路店）</t>
+          <t>希岸酒店河北玉田店</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>维也纳酒店(唐山丰润林荫路店)</t>
+          <t>希岸酒店(玉田店)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1589,13 +1589,13 @@
         <v>30</v>
       </c>
       <c r="O12" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P12" t="n">
         <v>30</v>
       </c>
       <c r="Q12" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R12" t="n">
         <v>30</v>
@@ -1635,17 +1635,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>7050678618342557730</t>
+          <t>7382896529226336271</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>IU酒店（唐山万达广场店）</t>
+          <t>维也纳酒店（唐山丰润林荫路店）</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>IU酒店(唐山万达广场店)</t>
+          <t>维也纳酒店(唐山丰润林荫路店)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -1671,7 +1671,7 @@
         <v>10</v>
       </c>
       <c r="M13" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N13" t="n">
         <v>30</v>
@@ -1683,7 +1683,7 @@
         <v>30</v>
       </c>
       <c r="Q13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R13" t="n">
         <v>30</v>
@@ -1723,17 +1723,17 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>7277808830371596324</t>
+          <t>7050678618342557730</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>河北省唐山市迁安市燕山中路项目</t>
+          <t>IU酒店（唐山万达广场店）</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>白玉兰酒店(迁安燕山中路店)</t>
+          <t>IU酒店(唐山万达广场店)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1759,19 +1759,19 @@
         <v>10</v>
       </c>
       <c r="M14" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N14" t="n">
         <v>30</v>
       </c>
       <c r="O14" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P14" t="n">
         <v>30</v>
       </c>
       <c r="Q14" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R14" t="n">
         <v>30</v>
@@ -1811,33 +1811,33 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>7405426591590828032</t>
+          <t>7277808830371596324</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>遵化燕山花园希岸Deluxe酒店</t>
+          <t>河北省唐山市迁安市燕山中路项目</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>遵化燕山花园希岸Deluxe酒店</t>
+          <t>白玉兰酒店(迁安燕山中路店)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>提质量,拿收益</t>
+          <t>稳房源,提质量,拿收益</t>
         </is>
       </c>
       <c r="K15" t="n">
@@ -1847,13 +1847,13 @@
         <v>10</v>
       </c>
       <c r="M15" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="N15" t="n">
         <v>30</v>
       </c>
       <c r="O15" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P15" t="n">
         <v>30</v>
@@ -1899,33 +1899,33 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>6740921212534327300</t>
+          <t>7405426591590828032</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>喆啡酒店（唐山遵化影大影城店）</t>
+          <t>遵化燕山花园希岸Deluxe酒店</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>喆啡酒店(遵化影大影城店)</t>
+          <t>遵化燕山花园希岸Deluxe酒店</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>稳房源,提质量,拿收益</t>
+          <t>提质量,拿收益</t>
         </is>
       </c>
       <c r="K16" t="n">
@@ -1935,19 +1935,19 @@
         <v>10</v>
       </c>
       <c r="M16" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="N16" t="n">
         <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P16" t="n">
         <v>30</v>
       </c>
       <c r="Q16" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R16" t="n">
         <v>30</v>
@@ -1987,17 +1987,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>6612824018124802055</t>
+          <t>6740921212534327300</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>7天优品（唐山迁西县政府店）</t>
+          <t>喆啡酒店（唐山遵化影大影城店）</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>7天优品酒店(迁西县政府店)</t>
+          <t>喆啡酒店(遵化影大影城店)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -2023,7 +2023,7 @@
         <v>10</v>
       </c>
       <c r="M17" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="N17" t="n">
         <v>30</v>
@@ -2075,17 +2075,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>7408054113827325978</t>
+          <t>6612824018124802055</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>IU酒店（唐山遵化长途汽车站店）</t>
+          <t>7天优品（唐山迁西县政府店）</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>IU酒店(唐山遵化长途汽车站店)</t>
+          <t>7天优品酒店(迁西县政府店)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2163,22 +2163,22 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>7318984134901925926</t>
+          <t>7408054113827325978</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>喆啡酒店（唐山万达广场国际五金城店）</t>
+          <t>IU酒店（唐山遵化长途汽车站店）</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>喆啡酒店(唐山万达广场国际五金城店)</t>
+          <t>IU酒店(唐山遵化长途汽车站店)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>提质量,拿收益</t>
+          <t>稳房源,提质量,拿收益</t>
         </is>
       </c>
       <c r="K19" t="n">
@@ -2199,7 +2199,7 @@
         <v>10</v>
       </c>
       <c r="M19" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N19" t="n">
         <v>30</v>
@@ -2211,7 +2211,7 @@
         <v>30</v>
       </c>
       <c r="Q19" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R19" t="n">
         <v>30</v>
@@ -2251,33 +2251,33 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>7236222858672752695</t>
+          <t>7318984134901925926</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>7天酒店（唐山丰润火车北站店）</t>
+          <t>喆啡酒店（唐山万达广场国际五金城店）</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>7天酒店(唐山丰润火车北站店)</t>
+          <t>喆啡酒店(唐山万达广场国际五金城店)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>稳房源,拿收益</t>
+          <t>提质量,拿收益</t>
         </is>
       </c>
       <c r="K20" t="n">
@@ -2287,19 +2287,19 @@
         <v>10</v>
       </c>
       <c r="M20" t="n">
+        <v>30</v>
+      </c>
+      <c r="N20" t="n">
+        <v>30</v>
+      </c>
+      <c r="O20" t="n">
         <v>25</v>
       </c>
-      <c r="N20" t="n">
-        <v>30</v>
-      </c>
-      <c r="O20" t="n">
-        <v>30</v>
-      </c>
       <c r="P20" t="n">
         <v>30</v>
       </c>
       <c r="Q20" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R20" t="n">
         <v>30</v>
@@ -2339,17 +2339,17 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>7325577924864641043</t>
+          <t>7236222858672752695</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>喆啡酒店（唐山爱琴海太阳城店）</t>
+          <t>7天酒店（唐山丰润火车北站店）</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>喆啡酒店(爱琴海太阳城店)</t>
+          <t>7天酒店(唐山丰润火车北站店)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>提质量,拿收益</t>
+          <t>稳房源,拿收益</t>
         </is>
       </c>
       <c r="K21" t="n">
@@ -2375,19 +2375,19 @@
         <v>10</v>
       </c>
       <c r="M21" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N21" t="n">
         <v>30</v>
       </c>
       <c r="O21" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P21" t="n">
         <v>30</v>
       </c>
       <c r="Q21" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="R21" t="n">
         <v>30</v>
@@ -2427,17 +2427,17 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>7495248853945075748</t>
+          <t>7325577924864641043</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>喆啡酒店（唐山会展中心师范学院店）</t>
+          <t>喆啡酒店（唐山爱琴海太阳城店）</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>喆啡酒店(唐山会展中心师范学院店)</t>
+          <t>喆啡酒店(爱琴海太阳城店)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2446,10 +2446,10 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="I22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         <v>30</v>
       </c>
       <c r="O22" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P22" t="n">
         <v>30</v>
@@ -2515,33 +2515,33 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>7278638524696365110</t>
+          <t>7495248853945075748</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>遵化文化南路锦江都城酒店</t>
+          <t>喆啡酒店（唐山会展中心师范学院店）</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>锦江都城酒店(遵化文化南路店)</t>
+          <t>喆啡酒店(唐山会展中心师范学院店)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H23" t="n">
         <v>110</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>拿收益</t>
+          <t>提质量,拿收益</t>
         </is>
       </c>
       <c r="K23" t="n">
@@ -2557,13 +2557,13 @@
         <v>30</v>
       </c>
       <c r="O23" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="P23" t="n">
         <v>30</v>
       </c>
       <c r="Q23" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R23" t="n">
         <v>30</v>
@@ -2603,22 +2603,22 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>6601148779653498888</t>
+          <t>7278638524696365110</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>锦江之星唐山人民医院小山酒店</t>
+          <t>遵化文化南路锦江都城酒店</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>锦江之星(唐山人民医院小山酒店)</t>
+          <t>锦江都城酒店(遵化文化南路店)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>稳房源,拿收益</t>
+          <t>拿收益</t>
         </is>
       </c>
       <c r="K24" t="n">
@@ -2639,7 +2639,7 @@
         <v>10</v>
       </c>
       <c r="M24" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="N24" t="n">
         <v>30</v>
@@ -2651,7 +2651,7 @@
         <v>30</v>
       </c>
       <c r="Q24" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="R24" t="n">
         <v>30</v>
@@ -2691,17 +2691,17 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>7239258071023749152</t>
+          <t>6601148779653498888</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>麗枫酒店（唐山世博广场万达店）</t>
+          <t>锦江之星唐山人民医院小山酒店</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>麗枫酒店(唐山世博广场万达店)</t>
+          <t>锦江之星(唐山人民医院小山酒店)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2713,11 +2713,11 @@
         <v>110</v>
       </c>
       <c r="I25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>提质量</t>
+          <t>稳房源,拿收益</t>
         </is>
       </c>
       <c r="K25" t="n">
@@ -2727,19 +2727,19 @@
         <v>10</v>
       </c>
       <c r="M25" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N25" t="n">
         <v>30</v>
       </c>
       <c r="O25" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P25" t="n">
         <v>30</v>
       </c>
       <c r="Q25" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="R25" t="n">
         <v>30</v>
@@ -2779,37 +2779,37 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>7561681153440188456</t>
+          <t>7239258071023749152</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>喆啡酒店（唐山玉田城市商业中心店）</t>
+          <t>麗枫酒店（唐山世博广场万达店）</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>喆啡酒店</t>
+          <t>麗枫酒店(唐山世博广场万达店)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I26" t="n">
         <v>5</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>搭门店,拿收益</t>
+          <t>提质量</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L26" t="n">
         <v>10</v>
@@ -2821,13 +2821,13 @@
         <v>30</v>
       </c>
       <c r="O26" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="P26" t="n">
         <v>30</v>
       </c>
       <c r="Q26" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="R26" t="n">
         <v>30</v>
@@ -2867,37 +2867,37 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>7497522879748933632</t>
+          <t>7561681153440188456</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>锦江之星（5.0唐山玉田无终西街旗舰酒店）</t>
+          <t>喆啡酒店（唐山玉田城市商业中心店）</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>锦江之星(唐山玉田无终西街旗舰酒店)</t>
+          <t>喆啡酒店</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>拿收益</t>
+          <t>搭门店,拿收益</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L27" t="n">
         <v>10</v>
@@ -2937,9 +2937,97 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>津河省区</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>唐山北片区</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>唐山市</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>7497522879748933632</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>锦江之星（5.0唐山玉田无终西街旗舰酒店）</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>锦江之星(唐山玉田无终西街旗舰酒店)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>已认证</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>115</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>拿收益</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>10</v>
+      </c>
+      <c r="L28" t="n">
+        <v>10</v>
+      </c>
+      <c r="M28" t="n">
+        <v>30</v>
+      </c>
+      <c r="N28" t="n">
+        <v>30</v>
+      </c>
+      <c r="O28" t="n">
+        <v>30</v>
+      </c>
+      <c r="P28" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>25</v>
+      </c>
+      <c r="R28" t="n">
+        <v>30</v>
+      </c>
+      <c r="S28" t="n">
+        <v>20</v>
+      </c>
+      <c r="T28" t="n">
+        <v>20</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>7249997748999555075</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>汇通百达网络科技（上海）有限公司</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V27"/>
-  <conditionalFormatting sqref="H2:H27">
+  <autoFilter ref="A1:V28"/>
+  <conditionalFormatting sqref="H2:H28">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2951,7 +3039,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I27">
+  <conditionalFormatting sqref="I2:I28">
     <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>